<commit_message>
docs(spec)+fixt: section 14.6c — the supply-status producers made normative (audit M5): the ref-level facts {openPO, overduePO, partialPO, supplierIssue} derived from live Open-POs lines against an explicit asOf; cancelled/closed lines leave the loop; banned-supplier is Supplier Issue; the Open-POs export gains Purchase Order Status (priority-1 ADD — template column provided, headers snapshot re-pinned, ingestion gap row added) — the contract text lands before the implementation, as the audit directive requires
</commit_message>
<xml_diff>
--- a/docs/templates/Sentinel_Ingestion_Template.xlsx
+++ b/docs/templates/Sentinel_Ingestion_Template.xlsx
@@ -1137,7 +1137,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -1158,7 +1158,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>OPEN POs — blue = verbatim "Open POs" headers. The standard export has NO creation date and NO price; add them to the Precoro export config or supply here, otherwise true lead time and price variance cannot be computed.</t>
+          <t>OPEN POs — blue = verbatim "Open POs" headers. The standard export has NO creation date, NO price and NO PO status; add them to the Precoro export config or supply here, otherwise true lead time and price variance cannot be computed.</t>
         </is>
       </c>
     </row>
@@ -1226,6 +1226,11 @@
       <c r="M2" s="2" t="inlineStr">
         <is>
           <t>Currency</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Purchase Order Status</t>
         </is>
       </c>
     </row>
@@ -1281,6 +1286,11 @@
           <t>BHD</t>
         </is>
       </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -1336,6 +1346,11 @@
       <c r="M4" t="inlineStr">
         <is>
           <t>BHD</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
         </is>
       </c>
     </row>
@@ -1591,7 +1606,6 @@
           <t>2026-08-30</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>Core</t>
@@ -1617,7 +1631,6 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>Core</t>

</xml_diff>